<commit_message>
ship: rebuild dictionary with page numbers
Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ship/dictionary.xlsx
+++ b/ship/dictionary.xlsx
@@ -63,13 +63,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -436,12 +439,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
     <col width="35" customWidth="1" min="2" max="2"/>
     <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -460,6 +464,11 @@
           <t>Deutsch</t>
         </is>
       </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Стр.</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -477,6 +486,9 @@
           <t>Konstruktionswasserlinie (KWL/OWL)</t>
         </is>
       </c>
+      <c r="D2" s="3" t="n">
+        <v>29</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -494,6 +506,9 @@
           <t>L\"ange \"uber Alles (LüA)</t>
         </is>
       </c>
+      <c r="D3" s="3" t="n">
+        <v>29</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -511,6 +526,9 @@
           <t>Beam \"uber Alles (BüA)</t>
         </is>
       </c>
+      <c r="D4" s="3" t="n">
+        <v>29</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -528,6 +546,9 @@
           <t>Tiefgang</t>
         </is>
       </c>
+      <c r="D5" s="3" t="n">
+        <v>29</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -544,6 +565,9 @@
         <is>
           <t>Verdr\"angung</t>
         </is>
+      </c>
+      <c r="D6" s="3" t="n">
+        <v>29</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
ch03: add pages 151-170 (sail form, aspect ratio, mast influence) + pics 103-115
Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ship/dictionary.xlsx
+++ b/ship/dictionary.xlsx
@@ -487,7 +487,7 @@
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="3">
@@ -507,7 +507,7 @@
         </is>
       </c>
       <c r="D3" s="3" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="4">
@@ -527,7 +527,7 @@
         </is>
       </c>
       <c r="D4" s="3" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="5">
@@ -547,7 +547,7 @@
         </is>
       </c>
       <c r="D5" s="3" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="6">
@@ -567,7 +567,7 @@
         </is>
       </c>
       <c r="D6" s="3" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
   </sheetData>

</xml_diff>